<commit_message>
Part 2- Easy & Medium tasks done with testing
</commit_message>
<xml_diff>
--- a/data/scenarios.xlsx
+++ b/data/scenarios.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="39">
   <si>
     <t>lap_number</t>
   </si>
@@ -55,151 +55,82 @@
     <t>medium</t>
   </si>
   <si>
-    <t>Low wear early in race. Stay out.</t>
-  </si>
-  <si>
-    <t>Healthy tyres. Stay out.</t>
-  </si>
-  <si>
-    <t>Moderate wear, still safe. Stay out.</t>
-  </si>
-  <si>
-    <t>Moderate wear. Stay out.</t>
-  </si>
-  <si>
-    <t>Wear increasing. Space behind allows conserving without losing position.</t>
-  </si>
-  <si>
-    <t>Getting high on wear, large gap allows conserving avoiding late pit.</t>
-  </si>
-  <si>
-    <t>Nearing end of race, conserve to survive to lap 30.</t>
-  </si>
-  <si>
-    <t>Tyres are good, gap is close. Push to overtake or undercut.</t>
-  </si>
-  <si>
-    <t>Tyres are fine, very close to car ahead. Push hard.</t>
-  </si>
-  <si>
-    <t>Tyre wear critical. Must pit to avoid failure.</t>
-  </si>
-  <si>
-    <t>Severe premature wear. Required pit.</t>
-  </si>
-  <si>
-    <t>Tyres about to explode. Pit immediately, even on last lap.</t>
-  </si>
-  <si>
-    <t>Borderline wear very early. Unsafe to continue. Pit.</t>
-  </si>
-  <si>
-    <t>Extremely close gap early. Push to pass.</t>
-  </si>
-  <si>
-    <t>Normal wear, nearing end. Stay out.</t>
-  </si>
-  <si>
-    <t>Cruising. Stay out.</t>
-  </si>
-  <si>
-    <t>Wear too high to risk to the end. Pit.</t>
-  </si>
-  <si>
-    <t>Decent wear but massive gap. Safely conserve tyres.</t>
-  </si>
-  <si>
-    <t>Good tyres, closing gap. Push.</t>
-  </si>
-  <si>
-    <t>Current tyres dry, weather rain. Must change strat.</t>
-  </si>
-  <si>
-    <t>High wear and rain. Perfect time to pit and swap to wets.</t>
-  </si>
-  <si>
-    <t>High wear but rain is coming. Conserve to drag out current tyres until rain hits to avoid double pit.</t>
-  </si>
-  <si>
-    <t>Tyres fine, gap tight. Stay out and wait for rain to pit.</t>
-  </si>
-  <si>
-    <t>Rain coming, but tyres are dead. Forced to pit now.</t>
-  </si>
-  <si>
-    <t>Borderline wear, but gap is tiny. Push to try and overtake before pitting.</t>
-  </si>
-  <si>
-    <t>High wear, normally a pit. But gap is close and race is almost over. Risk conserving.</t>
-  </si>
-  <si>
-    <t>Borderline wear, huge gap behind. Safe pit window available. Pit.</t>
-  </si>
-  <si>
-    <t>Moderate wear, close gap. Push to attack.</t>
-  </si>
-  <si>
-    <t>Moderate wear, large gap. No need to push, conserve.</t>
-  </si>
-  <si>
-    <t>Complex: Borderline wear, tight gap, rain imminent. Best to conserve and survive until rain hits to swap.</t>
-  </si>
-  <si>
-    <t>Rain hit late in race. Must change to wets to avoid crashing off track.</t>
-  </si>
-  <si>
-    <t>Early race, good tyres, close target. Push.</t>
-  </si>
-  <si>
-    <t>Tyres okay, large gap, rain coming. Stay out and hold position.</t>
-  </si>
-  <si>
-    <t>High wear and rain. Immediate swap required.</t>
-  </si>
-  <si>
-    <t>Middle of the road everything. Stay out.</t>
-  </si>
-  <si>
-    <t>Good tyres, awaiting rain. Stay out.</t>
-  </si>
-  <si>
-    <t>Too much wear. Pit.</t>
-  </si>
-  <si>
-    <t>Late race, wear getting high. Conserve to finish.</t>
-  </si>
-  <si>
-    <t>Fresh dry tyres but it started raining. Must swap.</t>
-  </si>
-  <si>
-    <t>High wear, but massive gap and rain coming. Conserve heavily to avoid two stops.</t>
-  </si>
-  <si>
-    <t>Very tight gap, good tyres. Maximum push.</t>
-  </si>
-  <si>
-    <t>Penultimate lap, close gap, but tyres critical. Must pit or DNF.</t>
-  </si>
-  <si>
-    <t>Raining. Irrelevant of gap, must swap tyres.</t>
-  </si>
-  <si>
-    <t>Late race wear management.</t>
-  </si>
-  <si>
-    <t>Tight battle, rain impending. Focus on staying out to swap on next lap.</t>
-  </si>
-  <si>
-    <t>Very tight gap overcut attempt but wear is too high to pull it off. Must pit.</t>
-  </si>
-  <si>
-    <t>Average situation. Stay out.</t>
-  </si>
-  <si>
-    <t>Solid lead, half wear. Safely conserve to finish.</t>
-  </si>
-  <si>
-    <t>Borderline wear, waiting for rain. Conserve.</t>
+    <t>R7: wear&lt;50, clear. Stay out.</t>
+  </si>
+  <si>
+    <t>R7: wear&lt;50, gap&gt;=2. Stay out.</t>
+  </si>
+  <si>
+    <t>R8: wear 50-60, clear. Stay out.</t>
+  </si>
+  <si>
+    <t>R5: wear 60-85, gap&gt;=5. Conserve.</t>
+  </si>
+  <si>
+    <t>R6: wear&lt;50, gap&lt;2. Push.</t>
+  </si>
+  <si>
+    <t>R2: wear&gt;=86. Pit immediately.</t>
+  </si>
+  <si>
+    <t>R2: wear&gt;=86. Pit.</t>
+  </si>
+  <si>
+    <t>R2: wear&gt;=86. Pit despite close gap.</t>
+  </si>
+  <si>
+    <t>R2: wear&gt;=86. Emergency pit.</t>
+  </si>
+  <si>
+    <t>R2: wear&gt;=86. Unsafe. Pit.</t>
+  </si>
+  <si>
+    <t>R1: rain. Swap immediately.</t>
+  </si>
+  <si>
+    <t>R1: rain. Swap.</t>
+  </si>
+  <si>
+    <t>R1: rain. Must swap.</t>
+  </si>
+  <si>
+    <t>R1: rain + high wear. Swap.</t>
+  </si>
+  <si>
+    <t>R1: rain. Swap urgently.</t>
+  </si>
+  <si>
+    <t>R1: rain. Gap irrelevant. Swap.</t>
+  </si>
+  <si>
+    <t>R2 beats R3: wear&gt;=86, pit now.</t>
+  </si>
+  <si>
+    <t>R2: wear&gt;=86. Pit or DNF.</t>
+  </si>
+  <si>
+    <t>R3: rain_soon, wear&gt;=70. Conserve.</t>
+  </si>
+  <si>
+    <t>R4: rain_soon, wear&lt;70. Stay out.</t>
+  </si>
+  <si>
+    <t>R5: clear, wear 60-85, gap&gt;=5. Conserve.</t>
+  </si>
+  <si>
+    <t>R5: late race, wear 60-85, gap&gt;=5. Conserve.</t>
+  </si>
+  <si>
+    <t>R6: wear&lt;50, gap&lt;2. Push hard.</t>
+  </si>
+  <si>
+    <t>R7: wear&lt;50, large gap. Stay out.</t>
+  </si>
+  <si>
+    <t>R3: wear&gt;=70, rain_soon. Conserve not pit.</t>
+  </si>
+  <si>
+    <t>R1: rain overrides everything. Swap.</t>
   </si>
 </sst>
 </file>
@@ -557,7 +488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -632,7 +563,7 @@
         <v>11</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>
@@ -658,7 +589,7 @@
         <v>11</v>
       </c>
       <c r="G4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -669,13 +600,13 @@
         <v>15</v>
       </c>
       <c r="B5">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -684,7 +615,7 @@
         <v>11</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H5" t="b">
         <v>0</v>
@@ -695,7 +626,7 @@
         <v>20</v>
       </c>
       <c r="B6">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C6" t="s">
         <v>8</v>
@@ -710,7 +641,7 @@
         <v>11</v>
       </c>
       <c r="G6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -718,25 +649,25 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B7">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
         <v>8</v>
       </c>
       <c r="D7">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F7" t="s">
         <v>11</v>
       </c>
       <c r="G7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H7" t="b">
         <v>0</v>
@@ -744,16 +675,16 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B8">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
         <v>8</v>
       </c>
       <c r="D8">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E8">
         <v>2</v>
@@ -762,7 +693,7 @@
         <v>11</v>
       </c>
       <c r="G8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -770,16 +701,16 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B9">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C9" t="s">
         <v>8</v>
       </c>
       <c r="D9">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -788,7 +719,7 @@
         <v>11</v>
       </c>
       <c r="G9" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="H9" t="b">
         <v>0</v>
@@ -796,25 +727,25 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="B10">
-        <v>30</v>
+        <v>75</v>
       </c>
       <c r="C10" t="s">
         <v>8</v>
       </c>
       <c r="D10">
-        <v>1.5</v>
+        <v>7</v>
       </c>
       <c r="E10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F10" t="s">
         <v>11</v>
       </c>
       <c r="G10" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -822,25 +753,25 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B11">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="C11" t="s">
         <v>8</v>
       </c>
       <c r="D11">
-        <v>0.8</v>
+        <v>20</v>
       </c>
       <c r="E11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F11" t="s">
         <v>11</v>
       </c>
       <c r="G11" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H11" t="b">
         <v>0</v>
@@ -848,51 +779,51 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B12">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
         <v>8</v>
       </c>
       <c r="D12">
-        <v>4</v>
+        <v>0.2</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F12" t="s">
         <v>11</v>
       </c>
       <c r="G12" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="H12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:8">
       <c r="A13">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B13">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
         <v>8</v>
       </c>
       <c r="D13">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F13" t="s">
         <v>11</v>
       </c>
       <c r="G13" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="H13" t="b">
         <v>0</v>
@@ -900,103 +831,103 @@
     </row>
     <row r="14" spans="1:8">
       <c r="A14">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B14">
-        <v>98</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
         <v>8</v>
       </c>
       <c r="D14">
-        <v>30</v>
+        <v>0.8</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F14" t="s">
         <v>11</v>
       </c>
       <c r="G14" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="H14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:8">
       <c r="A15">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="B15">
-        <v>78</v>
+        <v>48</v>
       </c>
       <c r="C15" t="s">
         <v>8</v>
       </c>
       <c r="D15">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F15" t="s">
         <v>11</v>
       </c>
       <c r="G15" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="H15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:8">
       <c r="A16">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="B16">
-        <v>15</v>
+        <v>86</v>
       </c>
       <c r="C16" t="s">
         <v>8</v>
       </c>
       <c r="D16">
-        <v>0.2</v>
+        <v>4</v>
       </c>
       <c r="E16">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F16" t="s">
         <v>11</v>
       </c>
       <c r="G16" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="H16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:8">
       <c r="A17">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="B17">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="C17" t="s">
         <v>8</v>
       </c>
       <c r="D17">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="E17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" t="s">
         <v>11</v>
       </c>
       <c r="G17" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H17" t="b">
         <v>0</v>
@@ -1004,42 +935,42 @@
     </row>
     <row r="18" spans="1:8">
       <c r="A18">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="B18">
-        <v>25</v>
+        <v>95</v>
       </c>
       <c r="C18" t="s">
         <v>8</v>
       </c>
       <c r="D18">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F18" t="s">
         <v>11</v>
       </c>
       <c r="G18" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="H18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:8">
       <c r="A19">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B19">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="C19" t="s">
         <v>8</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="E19">
         <v>0</v>
@@ -1048,59 +979,59 @@
         <v>11</v>
       </c>
       <c r="G19" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="H19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:8">
       <c r="A20">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B20">
-        <v>60</v>
+        <v>88</v>
       </c>
       <c r="C20" t="s">
         <v>8</v>
       </c>
       <c r="D20">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="E20">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F20" t="s">
         <v>11</v>
       </c>
       <c r="G20" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="H20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:8">
       <c r="A21">
+        <v>14</v>
+      </c>
+      <c r="B21">
+        <v>92</v>
+      </c>
+      <c r="C21" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21">
+        <v>5</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21" t="s">
+        <v>11</v>
+      </c>
+      <c r="G21" t="s">
         <v>19</v>
-      </c>
-      <c r="B21">
-        <v>35</v>
-      </c>
-      <c r="C21" t="s">
-        <v>8</v>
-      </c>
-      <c r="D21">
-        <v>1.2</v>
-      </c>
-      <c r="E21">
-        <v>3</v>
-      </c>
-      <c r="F21" t="s">
-        <v>11</v>
-      </c>
-      <c r="G21" t="s">
-        <v>31</v>
       </c>
       <c r="H21" t="b">
         <v>0</v>
@@ -1108,10 +1039,10 @@
     </row>
     <row r="22" spans="1:8">
       <c r="A22">
+        <v>5</v>
+      </c>
+      <c r="B22">
         <v>10</v>
-      </c>
-      <c r="B22">
-        <v>20</v>
       </c>
       <c r="C22" t="s">
         <v>9</v>
@@ -1126,7 +1057,7 @@
         <v>12</v>
       </c>
       <c r="G22" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="H22" t="b">
         <v>0</v>
@@ -1134,10 +1065,10 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B23">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="C23" t="s">
         <v>9</v>
@@ -1152,7 +1083,7 @@
         <v>12</v>
       </c>
       <c r="G23" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="H23" t="b">
         <v>0</v>
@@ -1160,25 +1091,25 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="B24">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="C24" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D24">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E24">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F24" t="s">
         <v>12</v>
       </c>
       <c r="G24" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="H24" t="b">
         <v>0</v>
@@ -1186,25 +1117,25 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B25">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="C25" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E25">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F25" t="s">
         <v>12</v>
       </c>
       <c r="G25" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="H25" t="b">
         <v>0</v>
@@ -1212,77 +1143,77 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="B26">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C26" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D26">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F26" t="s">
         <v>12</v>
       </c>
       <c r="G26" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="H26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:8">
       <c r="A27">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B27">
-        <v>75</v>
+        <v>40</v>
       </c>
       <c r="C27" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D27">
-        <v>0.5</v>
+        <v>15</v>
       </c>
       <c r="E27">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F27" t="s">
         <v>12</v>
       </c>
       <c r="G27" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="H27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:8">
       <c r="A28">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B28">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="C28" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D28">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E28">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F28" t="s">
         <v>12</v>
       </c>
       <c r="G28" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="H28" t="b">
         <v>1</v>
@@ -1290,16 +1221,16 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="B29">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="C29" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D29">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -1308,7 +1239,7 @@
         <v>12</v>
       </c>
       <c r="G29" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="H29" t="b">
         <v>1</v>
@@ -1316,25 +1247,25 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B30">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C30" t="s">
         <v>8</v>
       </c>
       <c r="D30">
-        <v>0.8</v>
+        <v>5</v>
       </c>
       <c r="E30">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F30" t="s">
         <v>12</v>
       </c>
       <c r="G30" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="H30" t="b">
         <v>0</v>
@@ -1342,42 +1273,42 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B31">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="C31" t="s">
         <v>8</v>
       </c>
       <c r="D31">
-        <v>15</v>
+        <v>0.5</v>
       </c>
       <c r="E31">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F31" t="s">
         <v>12</v>
       </c>
       <c r="G31" t="s">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="H31" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" spans="1:8">
       <c r="A32">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B32">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C32" t="s">
         <v>10</v>
       </c>
       <c r="D32">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="E32">
         <v>2</v>
@@ -1386,7 +1317,7 @@
         <v>12</v>
       </c>
       <c r="G32" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="H32" t="b">
         <v>0</v>
@@ -1394,77 +1325,77 @@
     </row>
     <row r="33" spans="1:8">
       <c r="A33">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="B33">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="C33" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D33">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E33">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F33" t="s">
         <v>12</v>
       </c>
       <c r="G33" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="H33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:8">
       <c r="A34">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="B34">
-        <v>15</v>
+        <v>80</v>
       </c>
       <c r="C34" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D34">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="E34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F34" t="s">
         <v>12</v>
       </c>
       <c r="G34" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="H34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:8">
       <c r="A35">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B35">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="C35" t="s">
         <v>10</v>
       </c>
       <c r="D35">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E35">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F35" t="s">
         <v>12</v>
       </c>
       <c r="G35" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="H35" t="b">
         <v>0</v>
@@ -1472,25 +1403,25 @@
     </row>
     <row r="36" spans="1:8">
       <c r="A36">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B36">
-        <v>90</v>
+        <v>40</v>
       </c>
       <c r="C36" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D36">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E36">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F36" t="s">
         <v>12</v>
       </c>
       <c r="G36" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="H36" t="b">
         <v>0</v>
@@ -1498,16 +1429,16 @@
     </row>
     <row r="37" spans="1:8">
       <c r="A37">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="B37">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="C37" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D37">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E37">
         <v>1</v>
@@ -1516,7 +1447,7 @@
         <v>12</v>
       </c>
       <c r="G37" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="H37" t="b">
         <v>0</v>
@@ -1524,16 +1455,16 @@
     </row>
     <row r="38" spans="1:8">
       <c r="A38">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="B38">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="C38" t="s">
         <v>10</v>
       </c>
       <c r="D38">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E38">
         <v>1</v>
@@ -1542,7 +1473,7 @@
         <v>12</v>
       </c>
       <c r="G38" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="H38" t="b">
         <v>0</v>
@@ -1550,25 +1481,25 @@
     </row>
     <row r="39" spans="1:8">
       <c r="A39">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B39">
-        <v>88</v>
+        <v>50</v>
       </c>
       <c r="C39" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D39">
-        <v>5</v>
+        <v>0.5</v>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F39" t="s">
         <v>12</v>
       </c>
       <c r="G39" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="H39" t="b">
         <v>0</v>
@@ -1576,16 +1507,16 @@
     </row>
     <row r="40" spans="1:8">
       <c r="A40">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="B40">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C40" t="s">
         <v>8</v>
       </c>
       <c r="D40">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E40">
         <v>2</v>
@@ -1594,7 +1525,7 @@
         <v>12</v>
       </c>
       <c r="G40" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="H40" t="b">
         <v>0</v>
@@ -1602,25 +1533,25 @@
     </row>
     <row r="41" spans="1:8">
       <c r="A41">
-        <v>5</v>
+        <v>26</v>
       </c>
       <c r="B41">
-        <v>10</v>
+        <v>70</v>
       </c>
       <c r="C41" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D41">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E41">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F41" t="s">
         <v>12</v>
       </c>
       <c r="G41" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="H41" t="b">
         <v>0</v>
@@ -1628,51 +1559,51 @@
     </row>
     <row r="42" spans="1:8">
       <c r="A42">
+        <v>24</v>
+      </c>
+      <c r="B42">
+        <v>74</v>
+      </c>
+      <c r="C42" t="s">
+        <v>8</v>
+      </c>
+      <c r="D42">
+        <v>2.5</v>
+      </c>
+      <c r="E42">
+        <v>2</v>
+      </c>
+      <c r="F42" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" t="s">
         <v>16</v>
       </c>
-      <c r="B42">
-        <v>81</v>
-      </c>
-      <c r="C42" t="s">
-        <v>10</v>
-      </c>
-      <c r="D42">
-        <v>20</v>
-      </c>
-      <c r="E42">
-        <v>2</v>
-      </c>
-      <c r="F42" t="s">
-        <v>12</v>
-      </c>
-      <c r="G42" t="s">
-        <v>52</v>
-      </c>
       <c r="H42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:8">
       <c r="A43">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="B43">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="C43" t="s">
         <v>8</v>
       </c>
       <c r="D43">
-        <v>0.3</v>
+        <v>8</v>
       </c>
       <c r="E43">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F43" t="s">
         <v>12</v>
       </c>
       <c r="G43" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="H43" t="b">
         <v>0</v>
@@ -1680,51 +1611,51 @@
     </row>
     <row r="44" spans="1:8">
       <c r="A44">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="B44">
-        <v>92</v>
+        <v>15</v>
       </c>
       <c r="C44" t="s">
         <v>8</v>
       </c>
       <c r="D44">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E44">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F44" t="s">
         <v>12</v>
       </c>
       <c r="G44" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="H44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:8">
       <c r="A45">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B45">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="C45" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D45">
-        <v>15</v>
+        <v>0.3</v>
       </c>
       <c r="E45">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F45" t="s">
         <v>12</v>
       </c>
       <c r="G45" t="s">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="H45" t="b">
         <v>0</v>
@@ -1732,25 +1663,25 @@
     </row>
     <row r="46" spans="1:8">
       <c r="A46">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B46">
-        <v>74</v>
+        <v>45</v>
       </c>
       <c r="C46" t="s">
         <v>8</v>
       </c>
       <c r="D46">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F46" t="s">
         <v>12</v>
       </c>
       <c r="G46" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="H46" t="b">
         <v>0</v>
@@ -1761,13 +1692,13 @@
         <v>18</v>
       </c>
       <c r="B47">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C47" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D47">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="E47">
         <v>1</v>
@@ -1776,7 +1707,7 @@
         <v>12</v>
       </c>
       <c r="G47" t="s">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="H47" t="b">
         <v>0</v>
@@ -1784,25 +1715,25 @@
     </row>
     <row r="48" spans="1:8">
       <c r="A48">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B48">
-        <v>85</v>
+        <v>45</v>
       </c>
       <c r="C48" t="s">
         <v>8</v>
       </c>
       <c r="D48">
-        <v>0.5</v>
+        <v>22</v>
       </c>
       <c r="E48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F48" t="s">
         <v>12</v>
       </c>
       <c r="G48" t="s">
-        <v>58</v>
+        <v>36</v>
       </c>
       <c r="H48" t="b">
         <v>0</v>
@@ -1810,80 +1741,54 @@
     </row>
     <row r="49" spans="1:8">
       <c r="A49">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B49">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="C49" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D49">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F49" t="s">
         <v>12</v>
       </c>
       <c r="G49" t="s">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="H49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:8">
       <c r="A50">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B50">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="C50" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D50">
-        <v>22</v>
+        <v>0.5</v>
       </c>
       <c r="E50">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F50" t="s">
         <v>12</v>
       </c>
       <c r="G50" t="s">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="H50" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8">
-      <c r="A51">
-        <v>19</v>
-      </c>
-      <c r="B51">
-        <v>72</v>
-      </c>
-      <c r="C51" t="s">
-        <v>10</v>
-      </c>
-      <c r="D51">
-        <v>4</v>
-      </c>
-      <c r="E51">
-        <v>2</v>
-      </c>
-      <c r="F51" t="s">
-        <v>12</v>
-      </c>
-      <c r="G51" t="s">
-        <v>61</v>
-      </c>
-      <c r="H51" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>